<commit_message>
feat: align import/export Excel sheet to exact 17-column layout and update template
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/Master Template.xlsx
+++ b/apps/web/public/templates/Master Template.xlsx
@@ -11,23 +11,23 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>TC ID</t>
   </si>
   <si>
+    <t>Menu</t>
+  </si>
+  <si>
+    <t>Scenario / Suite</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
     <t>Title</t>
   </si>
   <si>
-    <t>Sub-Module</t>
-  </si>
-  <si>
-    <t>Scenario</t>
-  </si>
-  <si>
-    <t>Type</t>
-  </si>
-  <si>
     <t>Severity</t>
   </si>
   <si>
@@ -37,9 +37,6 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Description</t>
-  </si>
-  <si>
     <t>Preconditions</t>
   </si>
   <si>
@@ -52,34 +49,19 @@
     <t>Actual Result</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Automation Status</t>
-  </si>
-  <si>
-    <t>Environment</t>
-  </si>
-  <si>
-    <t>Estimated Time</t>
-  </si>
-  <si>
-    <t>Requirement ID</t>
-  </si>
-  <si>
-    <t>Assigned To</t>
-  </si>
-  <si>
-    <t>Category</t>
+    <t>Notes / Evidence</t>
   </si>
   <si>
     <t>Author</t>
   </si>
   <si>
-    <t>Release Version</t>
-  </si>
-  <si>
-    <t>Is Automated</t>
+    <t>Date Created</t>
+  </si>
+  <si>
+    <t>Sprint / Release</t>
+  </si>
+  <si>
+    <t>Automation?</t>
   </si>
 </sst>
 </file>
@@ -479,31 +461,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="40" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="25" customWidth="1"/>
-    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="2" max="2" width="20" customWidth="1"/>
+    <col min="3" max="3" width="25" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
     <col min="6" max="7" width="12" customWidth="1"/>
     <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="32" customWidth="1"/>
-    <col min="10" max="10" width="28" customWidth="1"/>
-    <col min="11" max="11" width="45" customWidth="1"/>
-    <col min="12" max="13" width="38" customWidth="1"/>
-    <col min="14" max="14" width="24" customWidth="1"/>
-    <col min="15" max="15" width="20" customWidth="1"/>
-    <col min="16" max="17" width="15" customWidth="1"/>
-    <col min="18" max="18" width="18" customWidth="1"/>
-    <col min="19" max="19" width="20" customWidth="1"/>
-    <col min="20" max="20" width="14" customWidth="1"/>
-    <col min="21" max="22" width="18" customWidth="1"/>
-    <col min="23" max="23" width="14" customWidth="1"/>
+    <col min="9" max="9" width="28" customWidth="1"/>
+    <col min="10" max="10" width="45" customWidth="1"/>
+    <col min="11" max="12" width="38" customWidth="1"/>
+    <col min="13" max="13" width="24" customWidth="1"/>
+    <col min="14" max="16" width="18" customWidth="1"/>
+    <col min="17" max="17" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="1" ht="28" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -554,24 +530,6 @@
       </c>
       <c r="Q1" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: align Excel export/import with the styled 18-column grouped layout from references
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/Master Template.xlsx
+++ b/apps/web/public/templates/Master Template.xlsx
@@ -11,7 +11,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+  <si>
+    <t>Master Data — Test Cases</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
   <si>
     <t>TC ID</t>
   </si>
@@ -61,14 +67,14 @@
     <t>Sprint / Release</t>
   </si>
   <si>
-    <t>Automation?</t>
+    <t>Automated?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -79,16 +85,27 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
+      <sz val="12"/>
+      <name val="Inter"/>
+    </font>
+    <font>
+      <b/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
       <name val="Inter"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1E293B"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -105,9 +122,15 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
+      <left style="thin">
+        <color rgb="FF1E293B"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF1E293B"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF1E293B"/>
+      </top>
       <bottom style="medium">
         <color rgb="FF1E293B"/>
       </bottom>
@@ -117,9 +140,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -461,78 +487,109 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="14" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="25" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="40" customWidth="1"/>
-    <col min="6" max="7" width="12" customWidth="1"/>
-    <col min="8" max="8" width="14" customWidth="1"/>
-    <col min="9" max="9" width="28" customWidth="1"/>
-    <col min="10" max="10" width="45" customWidth="1"/>
-    <col min="11" max="12" width="38" customWidth="1"/>
-    <col min="13" max="13" width="24" customWidth="1"/>
-    <col min="14" max="16" width="18" customWidth="1"/>
-    <col min="17" max="17" width="14" customWidth="1"/>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="28" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="6" max="6" width="38" customWidth="1"/>
+    <col min="7" max="8" width="12" customWidth="1"/>
+    <col min="9" max="9" width="13" customWidth="1"/>
+    <col min="10" max="10" width="35" customWidth="1"/>
+    <col min="11" max="11" width="50" customWidth="1"/>
+    <col min="12" max="13" width="40" customWidth="1"/>
+    <col min="14" max="14" width="30" customWidth="1"/>
+    <col min="15" max="15" width="16" customWidth="1"/>
+    <col min="16" max="16" width="15" customWidth="1"/>
+    <col min="17" max="17" width="16" customWidth="1"/>
+    <col min="18" max="18" width="13" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" ht="40" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="F1" s="1"/>
+      <c r="G1" s="1"/>
+      <c r="H1" s="1"/>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+    </row>
+    <row r="2" ht="28" customHeight="1" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="E2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="F2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="G2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="I2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="J2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="K2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="L2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="M2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="N2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="O2" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="P2" s="2" t="s">
         <v>16</v>
+      </c>
+      <c r="Q2" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:R1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>